<commit_message>
Update gui fill invoices and udpate file payment_template
</commit_message>
<xml_diff>
--- a/MPR_Managerment/Templates/payment_template.xlsx
+++ b/MPR_Managerment/Templates/payment_template.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ERP_Final_Git\MPR_Managerment\Templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ERP_Final_Management\MPR_Managerment\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49C1CF5F-32D4-4996-82AC-49EC0AAF8ADF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F3E458C-9502-4CD3-BC9A-B5AD27D2A44E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{283D7EDF-6DA3-496F-9B09-7B30338ED4CA}"/>
+    <workbookView xWindow="-28920" yWindow="735" windowWidth="29040" windowHeight="15720" xr2:uid="{283D7EDF-6DA3-496F-9B09-7B30338ED4CA}"/>
   </bookViews>
   <sheets>
     <sheet name="PaymentRequset" sheetId="1" r:id="rId1"/>
@@ -1731,8 +1731,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="8">
-    <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="166" formatCode="_-&quot;₩&quot;* #,##0_-;\-&quot;₩&quot;* #,##0_-;_-&quot;₩&quot;* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="167" formatCode="0.00_ "/>
@@ -1744,14 +1744,14 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -1823,7 +1823,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <name val="Arial"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -1880,14 +1880,14 @@
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0">
@@ -1920,10 +1920,10 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="6" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="8" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1">
@@ -1959,116 +1959,116 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="6" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="5" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="13" fillId="0" borderId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="13" fillId="0" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="6" fillId="0" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="8" fillId="0" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="6" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -2094,70 +2094,6 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>0</xdr:col>
-          <xdr:colOff>47625</xdr:colOff>
-          <xdr:row>28</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>6</xdr:col>
-          <xdr:colOff>33619</xdr:colOff>
-          <xdr:row>31</xdr:row>
-          <xdr:rowOff>7844</xdr:rowOff>
-        </xdr:to>
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="2" name="Picture 1">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D4D01413-9BBF-43E4-83D4-CF1F1BFB8881}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr>
-              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-              <a:extLst>
-                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="#REF!" spid="_x0000_s1085"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPicPr>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-            <a:srcRect/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="47625" y="8998324"/>
-              <a:ext cx="3190876" cy="1868020"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:solidFill>
-              <a:srgbClr val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="9"/>
-            </a:solidFill>
-            <a:ln w="9525">
-              <a:noFill/>
-              <a:miter lim="800000"/>
-              <a:headEnd/>
-              <a:tailEnd/>
-            </a:ln>
-          </xdr:spPr>
-        </xdr:pic>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>15</xdr:col>
@@ -2204,6 +2140,50 @@
         </a:extLst>
       </xdr:spPr>
     </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>139212</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>227134</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>80597</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>100433</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8860C905-B1AE-9B7E-8E2A-7F683311B8B0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="139212" y="9048749"/>
+          <a:ext cx="3553558" cy="1741665"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -2532,57 +2512,57 @@
   <dimension ref="A1:O35"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="20.100000000000001" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="13.875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="2.125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="7.125" style="1" customWidth="1"/>
-    <col min="4" max="5" width="5.375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="8.25" style="1" customWidth="1"/>
+    <col min="1" max="1" width="13.85546875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="2.140625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="7.140625" style="1" customWidth="1"/>
+    <col min="4" max="5" width="5.42578125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" style="1" customWidth="1"/>
     <col min="7" max="7" width="12" style="1" customWidth="1"/>
-    <col min="8" max="8" width="4.25" style="1" customWidth="1"/>
-    <col min="9" max="10" width="4.375" style="1" customWidth="1"/>
-    <col min="11" max="11" width="1.875" style="1" customWidth="1"/>
-    <col min="12" max="12" width="1.375" style="1" customWidth="1"/>
-    <col min="13" max="13" width="10.375" style="1" customWidth="1"/>
-    <col min="14" max="14" width="13.875" style="1" customWidth="1"/>
-    <col min="15" max="15" width="24" style="58" customWidth="1"/>
+    <col min="8" max="8" width="4.28515625" style="1" customWidth="1"/>
+    <col min="9" max="10" width="4.42578125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="1.85546875" style="1" customWidth="1"/>
+    <col min="12" max="12" width="1.42578125" style="1" customWidth="1"/>
+    <col min="13" max="13" width="10.42578125" style="1" customWidth="1"/>
+    <col min="14" max="14" width="13.85546875" style="1" customWidth="1"/>
+    <col min="15" max="15" width="24" style="25" customWidth="1"/>
     <col min="16" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="30" customHeight="1">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="54" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-      <c r="K1" s="23"/>
-      <c r="L1" s="23"/>
-      <c r="M1" s="23"/>
-      <c r="N1" s="23"/>
-      <c r="O1" s="23"/>
+      <c r="B1" s="55"/>
+      <c r="C1" s="55"/>
+      <c r="D1" s="55"/>
+      <c r="E1" s="55"/>
+      <c r="F1" s="55"/>
+      <c r="G1" s="55"/>
+      <c r="H1" s="55"/>
+      <c r="I1" s="55"/>
+      <c r="J1" s="55"/>
+      <c r="K1" s="55"/>
+      <c r="L1" s="55"/>
+      <c r="M1" s="55"/>
+      <c r="N1" s="55"/>
+      <c r="O1" s="55"/>
     </row>
     <row r="2" spans="1:15" s="4" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A2" s="24"/>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-      <c r="I2" s="24"/>
-      <c r="J2" s="24"/>
-      <c r="K2" s="24"/>
-      <c r="L2" s="24"/>
-      <c r="M2" s="24"/>
-      <c r="N2" s="24"/>
-      <c r="O2" s="24"/>
+      <c r="A2" s="26"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
+      <c r="I2" s="26"/>
+      <c r="J2" s="26"/>
+      <c r="K2" s="26"/>
+      <c r="L2" s="26"/>
+      <c r="M2" s="26"/>
+      <c r="N2" s="26"/>
+      <c r="O2" s="26"/>
     </row>
     <row r="3" spans="1:15" s="4" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A3" s="6" t="s">
@@ -2591,19 +2571,19 @@
       <c r="B3" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="25"/>
-      <c r="D3" s="26"/>
-      <c r="E3" s="26"/>
-      <c r="F3" s="26"/>
-      <c r="G3" s="26"/>
-      <c r="H3" s="26"/>
-      <c r="I3" s="26"/>
-      <c r="J3" s="26"/>
-      <c r="K3" s="26"/>
-      <c r="L3" s="26"/>
-      <c r="M3" s="26"/>
-      <c r="N3" s="26"/>
-      <c r="O3" s="26"/>
+      <c r="C3" s="56"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="57"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="57"/>
+      <c r="L3" s="57"/>
+      <c r="M3" s="57"/>
+      <c r="N3" s="57"/>
+      <c r="O3" s="57"/>
     </row>
     <row r="4" spans="1:15" s="4" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A4" s="6" t="s">
@@ -2612,19 +2592,19 @@
       <c r="B4" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="25"/>
-      <c r="D4" s="26"/>
-      <c r="E4" s="26"/>
-      <c r="F4" s="26"/>
-      <c r="G4" s="26"/>
-      <c r="H4" s="26"/>
-      <c r="I4" s="26"/>
-      <c r="J4" s="26"/>
-      <c r="K4" s="26"/>
-      <c r="L4" s="26"/>
-      <c r="M4" s="26"/>
-      <c r="N4" s="26"/>
-      <c r="O4" s="26"/>
+      <c r="C4" s="56"/>
+      <c r="D4" s="57"/>
+      <c r="E4" s="57"/>
+      <c r="F4" s="57"/>
+      <c r="G4" s="57"/>
+      <c r="H4" s="57"/>
+      <c r="I4" s="57"/>
+      <c r="J4" s="57"/>
+      <c r="K4" s="57"/>
+      <c r="L4" s="57"/>
+      <c r="M4" s="57"/>
+      <c r="N4" s="57"/>
+      <c r="O4" s="57"/>
     </row>
     <row r="5" spans="1:15" s="4" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A5" s="6" t="s">
@@ -2633,27 +2613,27 @@
       <c r="B5" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="24" t="s">
+      <c r="C5" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="D5" s="24"/>
-      <c r="E5" s="24"/>
-      <c r="F5" s="24"/>
-      <c r="G5" s="24"/>
-      <c r="H5" s="24"/>
-      <c r="I5" s="27" t="s">
+      <c r="D5" s="26"/>
+      <c r="E5" s="26"/>
+      <c r="F5" s="26"/>
+      <c r="G5" s="26"/>
+      <c r="H5" s="26"/>
+      <c r="I5" s="47" t="s">
         <v>7</v>
       </c>
-      <c r="J5" s="27"/>
-      <c r="K5" s="27"/>
+      <c r="J5" s="47"/>
+      <c r="K5" s="47"/>
       <c r="L5" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="M5" s="28" t="s">
+      <c r="M5" s="58" t="s">
         <v>34</v>
       </c>
-      <c r="N5" s="28"/>
-      <c r="O5" s="28"/>
+      <c r="N5" s="58"/>
+      <c r="O5" s="58"/>
     </row>
     <row r="6" spans="1:15" s="4" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A6" s="6" t="s">
@@ -2662,25 +2642,25 @@
       <c r="B6" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="31" t="s">
+      <c r="C6" s="45" t="s">
         <v>60</v>
       </c>
-      <c r="D6" s="32"/>
-      <c r="E6" s="32"/>
-      <c r="F6" s="32"/>
-      <c r="G6" s="32"/>
-      <c r="H6" s="32"/>
-      <c r="I6" s="27" t="s">
+      <c r="D6" s="46"/>
+      <c r="E6" s="46"/>
+      <c r="F6" s="46"/>
+      <c r="G6" s="46"/>
+      <c r="H6" s="46"/>
+      <c r="I6" s="47" t="s">
         <v>9</v>
       </c>
-      <c r="J6" s="27"/>
-      <c r="K6" s="27"/>
+      <c r="J6" s="47"/>
+      <c r="K6" s="47"/>
       <c r="L6" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="M6" s="33"/>
-      <c r="N6" s="33"/>
-      <c r="O6" s="33"/>
+      <c r="M6" s="48"/>
+      <c r="N6" s="48"/>
+      <c r="O6" s="48"/>
     </row>
     <row r="7" spans="1:15" s="4" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A7" s="6" t="s">
@@ -2689,25 +2669,25 @@
       <c r="B7" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="34" t="s">
+      <c r="C7" s="49" t="s">
         <v>39</v>
       </c>
-      <c r="D7" s="35"/>
-      <c r="E7" s="35"/>
-      <c r="F7" s="35"/>
-      <c r="G7" s="35"/>
-      <c r="H7" s="35"/>
-      <c r="I7" s="36" t="s">
+      <c r="D7" s="50"/>
+      <c r="E7" s="50"/>
+      <c r="F7" s="50"/>
+      <c r="G7" s="50"/>
+      <c r="H7" s="50"/>
+      <c r="I7" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="J7" s="36"/>
+      <c r="J7" s="33"/>
       <c r="K7" s="9"/>
-      <c r="L7" s="37" t="s">
+      <c r="L7" s="51" t="s">
         <v>12</v>
       </c>
-      <c r="M7" s="37"/>
-      <c r="N7" s="37"/>
-      <c r="O7" s="55"/>
+      <c r="M7" s="51"/>
+      <c r="N7" s="51"/>
+      <c r="O7" s="22"/>
     </row>
     <row r="8" spans="1:15" s="11" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A8" s="6" t="s">
@@ -2716,25 +2696,25 @@
       <c r="B8" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C8" s="34" t="s">
+      <c r="C8" s="49" t="s">
         <v>36</v>
       </c>
-      <c r="D8" s="35"/>
-      <c r="E8" s="35"/>
-      <c r="F8" s="35"/>
-      <c r="G8" s="35"/>
-      <c r="H8" s="35"/>
-      <c r="I8" s="36" t="s">
+      <c r="D8" s="50"/>
+      <c r="E8" s="50"/>
+      <c r="F8" s="50"/>
+      <c r="G8" s="50"/>
+      <c r="H8" s="50"/>
+      <c r="I8" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="J8" s="36"/>
+      <c r="J8" s="33"/>
       <c r="K8" s="10"/>
-      <c r="L8" s="38" t="s">
+      <c r="L8" s="52" t="s">
         <v>12</v>
       </c>
-      <c r="M8" s="38"/>
-      <c r="N8" s="38"/>
-      <c r="O8" s="56"/>
+      <c r="M8" s="52"/>
+      <c r="N8" s="52"/>
+      <c r="O8" s="23"/>
     </row>
     <row r="9" spans="1:15" s="4" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A9" s="6" t="s">
@@ -2743,63 +2723,63 @@
       <c r="B9" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C9" s="36" t="s">
+      <c r="C9" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="36"/>
-      <c r="E9" s="36"/>
-      <c r="F9" s="36"/>
-      <c r="G9" s="36"/>
-      <c r="H9" s="36"/>
-      <c r="I9" s="36"/>
-      <c r="J9" s="36"/>
-      <c r="K9" s="36"/>
-      <c r="L9" s="36"/>
-      <c r="M9" s="36"/>
-      <c r="N9" s="36"/>
-      <c r="O9" s="36"/>
+      <c r="D9" s="33"/>
+      <c r="E9" s="33"/>
+      <c r="F9" s="33"/>
+      <c r="G9" s="33"/>
+      <c r="H9" s="33"/>
+      <c r="I9" s="33"/>
+      <c r="J9" s="33"/>
+      <c r="K9" s="33"/>
+      <c r="L9" s="33"/>
+      <c r="M9" s="33"/>
+      <c r="N9" s="33"/>
+      <c r="O9" s="33"/>
     </row>
     <row r="10" spans="1:15" s="4" customFormat="1" ht="5.0999999999999996" customHeight="1">
-      <c r="A10" s="39"/>
-      <c r="B10" s="39"/>
-      <c r="C10" s="39"/>
-      <c r="D10" s="39"/>
-      <c r="E10" s="39"/>
-      <c r="F10" s="39"/>
-      <c r="G10" s="39"/>
-      <c r="H10" s="39"/>
-      <c r="I10" s="39"/>
-      <c r="J10" s="39"/>
-      <c r="K10" s="39"/>
-      <c r="L10" s="39"/>
-      <c r="M10" s="39"/>
-      <c r="N10" s="39"/>
-      <c r="O10" s="39"/>
+      <c r="A10" s="53"/>
+      <c r="B10" s="53"/>
+      <c r="C10" s="53"/>
+      <c r="D10" s="53"/>
+      <c r="E10" s="53"/>
+      <c r="F10" s="53"/>
+      <c r="G10" s="53"/>
+      <c r="H10" s="53"/>
+      <c r="I10" s="53"/>
+      <c r="J10" s="53"/>
+      <c r="K10" s="53"/>
+      <c r="L10" s="53"/>
+      <c r="M10" s="53"/>
+      <c r="N10" s="53"/>
+      <c r="O10" s="53"/>
     </row>
     <row r="11" spans="1:15" s="3" customFormat="1" ht="30" customHeight="1">
       <c r="A11" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="29" t="s">
+      <c r="B11" s="43" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="30"/>
-      <c r="D11" s="30"/>
-      <c r="E11" s="30"/>
-      <c r="F11" s="30" t="s">
+      <c r="C11" s="44"/>
+      <c r="D11" s="44"/>
+      <c r="E11" s="44"/>
+      <c r="F11" s="44" t="s">
         <v>18</v>
       </c>
-      <c r="G11" s="30"/>
-      <c r="H11" s="30" t="s">
+      <c r="G11" s="44"/>
+      <c r="H11" s="44" t="s">
         <v>19</v>
       </c>
-      <c r="I11" s="30"/>
-      <c r="J11" s="30"/>
-      <c r="K11" s="30"/>
-      <c r="L11" s="29" t="s">
+      <c r="I11" s="44"/>
+      <c r="J11" s="44"/>
+      <c r="K11" s="44"/>
+      <c r="L11" s="43" t="s">
         <v>20</v>
       </c>
-      <c r="M11" s="30"/>
+      <c r="M11" s="44"/>
       <c r="N11" s="12" t="s">
         <v>21</v>
       </c>
@@ -2811,136 +2791,136 @@
       <c r="A12" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B12" s="40" t="s">
+      <c r="B12" s="35" t="s">
         <v>37</v>
       </c>
-      <c r="C12" s="40"/>
-      <c r="D12" s="40"/>
-      <c r="E12" s="40"/>
-      <c r="F12" s="41" t="s">
+      <c r="C12" s="35"/>
+      <c r="D12" s="35"/>
+      <c r="E12" s="35"/>
+      <c r="F12" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="G12" s="42"/>
-      <c r="H12" s="42" t="s">
+      <c r="G12" s="37"/>
+      <c r="H12" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="I12" s="42"/>
-      <c r="J12" s="42"/>
-      <c r="K12" s="42"/>
-      <c r="L12" s="43"/>
-      <c r="M12" s="44"/>
+      <c r="I12" s="37"/>
+      <c r="J12" s="37"/>
+      <c r="K12" s="37"/>
+      <c r="L12" s="41"/>
+      <c r="M12" s="42"/>
       <c r="N12" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="O12" s="57"/>
+      <c r="O12" s="24"/>
     </row>
     <row r="13" spans="1:15" s="4" customFormat="1" ht="24.95" customHeight="1">
       <c r="A13" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="B13" s="40" t="s">
+      <c r="B13" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="C13" s="40"/>
-      <c r="D13" s="40"/>
-      <c r="E13" s="40"/>
-      <c r="F13" s="41" t="s">
+      <c r="C13" s="35"/>
+      <c r="D13" s="35"/>
+      <c r="E13" s="35"/>
+      <c r="F13" s="36" t="s">
         <v>46</v>
       </c>
-      <c r="G13" s="42"/>
-      <c r="H13" s="42" t="s">
+      <c r="G13" s="37"/>
+      <c r="H13" s="37" t="s">
         <v>50</v>
       </c>
-      <c r="I13" s="42"/>
-      <c r="J13" s="42"/>
-      <c r="K13" s="42"/>
-      <c r="L13" s="45"/>
-      <c r="M13" s="45"/>
+      <c r="I13" s="37"/>
+      <c r="J13" s="37"/>
+      <c r="K13" s="37"/>
+      <c r="L13" s="38"/>
+      <c r="M13" s="38"/>
       <c r="N13" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="O13" s="57"/>
+      <c r="O13" s="24"/>
     </row>
     <row r="14" spans="1:15" s="4" customFormat="1" ht="24.95" customHeight="1">
       <c r="A14" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="40" t="s">
+      <c r="B14" s="35" t="s">
         <v>43</v>
       </c>
-      <c r="C14" s="40"/>
-      <c r="D14" s="40"/>
-      <c r="E14" s="40"/>
-      <c r="F14" s="41" t="s">
+      <c r="C14" s="35"/>
+      <c r="D14" s="35"/>
+      <c r="E14" s="35"/>
+      <c r="F14" s="36" t="s">
         <v>47</v>
       </c>
-      <c r="G14" s="42"/>
-      <c r="H14" s="42" t="s">
+      <c r="G14" s="37"/>
+      <c r="H14" s="37" t="s">
         <v>51</v>
       </c>
-      <c r="I14" s="42"/>
-      <c r="J14" s="42"/>
-      <c r="K14" s="42"/>
-      <c r="L14" s="45"/>
-      <c r="M14" s="45"/>
+      <c r="I14" s="37"/>
+      <c r="J14" s="37"/>
+      <c r="K14" s="37"/>
+      <c r="L14" s="38"/>
+      <c r="M14" s="38"/>
       <c r="N14" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="O14" s="57"/>
+      <c r="O14" s="24"/>
     </row>
     <row r="15" spans="1:15" s="4" customFormat="1" ht="24.95" customHeight="1">
       <c r="A15" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="B15" s="40" t="s">
+      <c r="B15" s="35" t="s">
         <v>44</v>
       </c>
-      <c r="C15" s="40"/>
-      <c r="D15" s="40"/>
-      <c r="E15" s="40"/>
-      <c r="F15" s="41" t="s">
+      <c r="C15" s="35"/>
+      <c r="D15" s="35"/>
+      <c r="E15" s="35"/>
+      <c r="F15" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="G15" s="42"/>
-      <c r="H15" s="42" t="s">
+      <c r="G15" s="37"/>
+      <c r="H15" s="37" t="s">
         <v>52</v>
       </c>
-      <c r="I15" s="42"/>
-      <c r="J15" s="42"/>
-      <c r="K15" s="42"/>
-      <c r="L15" s="45"/>
-      <c r="M15" s="45"/>
+      <c r="I15" s="37"/>
+      <c r="J15" s="37"/>
+      <c r="K15" s="37"/>
+      <c r="L15" s="38"/>
+      <c r="M15" s="38"/>
       <c r="N15" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="O15" s="57"/>
+      <c r="O15" s="24"/>
     </row>
     <row r="16" spans="1:15" s="4" customFormat="1" ht="24.95" customHeight="1">
       <c r="A16" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="40" t="s">
+      <c r="B16" s="35" t="s">
         <v>45</v>
       </c>
-      <c r="C16" s="40"/>
-      <c r="D16" s="40"/>
-      <c r="E16" s="40"/>
-      <c r="F16" s="41" t="s">
+      <c r="C16" s="35"/>
+      <c r="D16" s="35"/>
+      <c r="E16" s="35"/>
+      <c r="F16" s="36" t="s">
         <v>49</v>
       </c>
-      <c r="G16" s="42"/>
-      <c r="H16" s="42" t="s">
+      <c r="G16" s="37"/>
+      <c r="H16" s="37" t="s">
         <v>53</v>
       </c>
-      <c r="I16" s="42"/>
-      <c r="J16" s="42"/>
-      <c r="K16" s="42"/>
-      <c r="L16" s="45"/>
-      <c r="M16" s="45"/>
+      <c r="I16" s="37"/>
+      <c r="J16" s="37"/>
+      <c r="K16" s="37"/>
+      <c r="L16" s="38"/>
+      <c r="M16" s="38"/>
       <c r="N16" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="O16" s="57"/>
+      <c r="O16" s="24"/>
     </row>
     <row r="17" spans="1:15" s="4" customFormat="1" ht="24.95" hidden="1" customHeight="1">
       <c r="A17" s="8"/>
@@ -2957,218 +2937,218 @@
       <c r="L17" s="19"/>
       <c r="M17" s="19"/>
       <c r="N17" s="18"/>
-      <c r="O17" s="57"/>
+      <c r="O17" s="24"/>
     </row>
     <row r="18" spans="1:15" s="4" customFormat="1" ht="24.95" customHeight="1">
       <c r="A18" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B18" s="46" t="s">
+      <c r="B18" s="39" t="s">
         <v>38</v>
       </c>
-      <c r="C18" s="46"/>
-      <c r="D18" s="46"/>
-      <c r="E18" s="46"/>
-      <c r="F18" s="42" t="s">
+      <c r="C18" s="39"/>
+      <c r="D18" s="39"/>
+      <c r="E18" s="39"/>
+      <c r="F18" s="37" t="s">
         <v>38</v>
       </c>
-      <c r="G18" s="42"/>
-      <c r="H18" s="42" t="s">
+      <c r="G18" s="37"/>
+      <c r="H18" s="37" t="s">
         <v>38</v>
       </c>
-      <c r="I18" s="42"/>
-      <c r="J18" s="42"/>
-      <c r="K18" s="42"/>
-      <c r="L18" s="45"/>
-      <c r="M18" s="45"/>
+      <c r="I18" s="37"/>
+      <c r="J18" s="37"/>
+      <c r="K18" s="37"/>
+      <c r="L18" s="38"/>
+      <c r="M18" s="38"/>
       <c r="N18" s="20"/>
-      <c r="O18" s="57"/>
+      <c r="O18" s="24"/>
     </row>
     <row r="19" spans="1:15" s="4" customFormat="1" ht="35.25" customHeight="1">
       <c r="A19" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="B19" s="47" t="s">
+      <c r="B19" s="40" t="s">
         <v>59</v>
       </c>
-      <c r="C19" s="47"/>
-      <c r="D19" s="47"/>
-      <c r="E19" s="47"/>
-      <c r="F19" s="41"/>
-      <c r="G19" s="42"/>
-      <c r="H19" s="42" t="s">
+      <c r="C19" s="40"/>
+      <c r="D19" s="40"/>
+      <c r="E19" s="40"/>
+      <c r="F19" s="36"/>
+      <c r="G19" s="37"/>
+      <c r="H19" s="37" t="s">
         <v>54</v>
       </c>
-      <c r="I19" s="42"/>
-      <c r="J19" s="42"/>
-      <c r="K19" s="42"/>
-      <c r="L19" s="45"/>
-      <c r="M19" s="45"/>
+      <c r="I19" s="37"/>
+      <c r="J19" s="37"/>
+      <c r="K19" s="37"/>
+      <c r="L19" s="38"/>
+      <c r="M19" s="38"/>
       <c r="N19" s="20"/>
-      <c r="O19" s="57"/>
+      <c r="O19" s="24"/>
     </row>
     <row r="20" spans="1:15" s="4" customFormat="1" ht="18" customHeight="1">
-      <c r="A20" s="24"/>
-      <c r="B20" s="24"/>
-      <c r="C20" s="24"/>
-      <c r="D20" s="24"/>
-      <c r="E20" s="24"/>
-      <c r="F20" s="24"/>
-      <c r="G20" s="24"/>
-      <c r="H20" s="24"/>
-      <c r="I20" s="24"/>
-      <c r="J20" s="24"/>
-      <c r="K20" s="24"/>
-      <c r="L20" s="24"/>
-      <c r="M20" s="24"/>
-      <c r="N20" s="24"/>
-      <c r="O20" s="24"/>
+      <c r="A20" s="26"/>
+      <c r="B20" s="26"/>
+      <c r="C20" s="26"/>
+      <c r="D20" s="26"/>
+      <c r="E20" s="26"/>
+      <c r="F20" s="26"/>
+      <c r="G20" s="26"/>
+      <c r="H20" s="26"/>
+      <c r="I20" s="26"/>
+      <c r="J20" s="26"/>
+      <c r="K20" s="26"/>
+      <c r="L20" s="26"/>
+      <c r="M20" s="26"/>
+      <c r="N20" s="26"/>
+      <c r="O20" s="26"/>
     </row>
     <row r="21" spans="1:15" s="4" customFormat="1" ht="18" customHeight="1">
-      <c r="A21" s="36" t="s">
+      <c r="A21" s="33" t="s">
         <v>28</v>
       </c>
-      <c r="B21" s="36"/>
-      <c r="C21" s="36"/>
-      <c r="D21" s="36"/>
-      <c r="E21" s="36"/>
-      <c r="F21" s="36"/>
-      <c r="G21" s="36"/>
-      <c r="H21" s="36"/>
-      <c r="I21" s="36"/>
-      <c r="J21" s="36"/>
-      <c r="K21" s="36"/>
-      <c r="L21" s="36"/>
-      <c r="M21" s="36"/>
-      <c r="N21" s="36"/>
-      <c r="O21" s="36"/>
+      <c r="B21" s="33"/>
+      <c r="C21" s="33"/>
+      <c r="D21" s="33"/>
+      <c r="E21" s="33"/>
+      <c r="F21" s="33"/>
+      <c r="G21" s="33"/>
+      <c r="H21" s="33"/>
+      <c r="I21" s="33"/>
+      <c r="J21" s="33"/>
+      <c r="K21" s="33"/>
+      <c r="L21" s="33"/>
+      <c r="M21" s="33"/>
+      <c r="N21" s="33"/>
+      <c r="O21" s="33"/>
     </row>
     <row r="22" spans="1:15" s="4" customFormat="1" ht="18" customHeight="1">
-      <c r="A22" s="36" t="s">
+      <c r="A22" s="33" t="s">
         <v>29</v>
       </c>
-      <c r="B22" s="36"/>
-      <c r="C22" s="36"/>
-      <c r="D22" s="36"/>
-      <c r="E22" s="36"/>
-      <c r="F22" s="36"/>
-      <c r="G22" s="36"/>
-      <c r="H22" s="36"/>
-      <c r="I22" s="36"/>
-      <c r="J22" s="36"/>
-      <c r="K22" s="36"/>
-      <c r="L22" s="36"/>
-      <c r="M22" s="36"/>
-      <c r="N22" s="36"/>
-      <c r="O22" s="36"/>
+      <c r="B22" s="33"/>
+      <c r="C22" s="33"/>
+      <c r="D22" s="33"/>
+      <c r="E22" s="33"/>
+      <c r="F22" s="33"/>
+      <c r="G22" s="33"/>
+      <c r="H22" s="33"/>
+      <c r="I22" s="33"/>
+      <c r="J22" s="33"/>
+      <c r="K22" s="33"/>
+      <c r="L22" s="33"/>
+      <c r="M22" s="33"/>
+      <c r="N22" s="33"/>
+      <c r="O22" s="33"/>
     </row>
     <row r="23" spans="1:15" s="4" customFormat="1" ht="18" customHeight="1">
-      <c r="A23" s="24"/>
-      <c r="B23" s="24"/>
-      <c r="C23" s="24"/>
-      <c r="D23" s="24"/>
-      <c r="E23" s="24"/>
-      <c r="F23" s="24"/>
-      <c r="G23" s="24"/>
-      <c r="H23" s="24"/>
-      <c r="I23" s="24"/>
-      <c r="J23" s="24"/>
-      <c r="K23" s="24"/>
-      <c r="L23" s="24"/>
-      <c r="M23" s="24"/>
-      <c r="N23" s="24"/>
-      <c r="O23" s="24"/>
+      <c r="A23" s="26"/>
+      <c r="B23" s="26"/>
+      <c r="C23" s="26"/>
+      <c r="D23" s="26"/>
+      <c r="E23" s="26"/>
+      <c r="F23" s="26"/>
+      <c r="G23" s="26"/>
+      <c r="H23" s="26"/>
+      <c r="I23" s="26"/>
+      <c r="J23" s="26"/>
+      <c r="K23" s="26"/>
+      <c r="L23" s="26"/>
+      <c r="M23" s="26"/>
+      <c r="N23" s="26"/>
+      <c r="O23" s="26"/>
     </row>
     <row r="24" spans="1:15" s="4" customFormat="1" ht="18" customHeight="1">
-      <c r="A24" s="51" t="s">
+      <c r="A24" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="B24" s="51"/>
-      <c r="C24" s="51"/>
-      <c r="D24" s="51"/>
-      <c r="E24" s="51"/>
-      <c r="F24" s="51"/>
-      <c r="G24" s="51"/>
-      <c r="H24" s="51"/>
-      <c r="I24" s="51"/>
-      <c r="J24" s="51"/>
-      <c r="K24" s="51"/>
-      <c r="L24" s="51"/>
-      <c r="M24" s="51"/>
-      <c r="N24" s="51"/>
-      <c r="O24" s="51"/>
+      <c r="B24" s="28"/>
+      <c r="C24" s="28"/>
+      <c r="D24" s="28"/>
+      <c r="E24" s="28"/>
+      <c r="F24" s="28"/>
+      <c r="G24" s="28"/>
+      <c r="H24" s="28"/>
+      <c r="I24" s="28"/>
+      <c r="J24" s="28"/>
+      <c r="K24" s="28"/>
+      <c r="L24" s="28"/>
+      <c r="M24" s="28"/>
+      <c r="N24" s="28"/>
+      <c r="O24" s="28"/>
     </row>
     <row r="25" spans="1:15" s="4" customFormat="1" ht="18" customHeight="1">
-      <c r="A25" s="51"/>
-      <c r="B25" s="51"/>
-      <c r="C25" s="51"/>
-      <c r="D25" s="51"/>
-      <c r="E25" s="51"/>
-      <c r="F25" s="51"/>
-      <c r="G25" s="51"/>
-      <c r="H25" s="51"/>
-      <c r="I25" s="51"/>
-      <c r="J25" s="51"/>
-      <c r="K25" s="51"/>
-      <c r="L25" s="51"/>
-      <c r="M25" s="51"/>
-      <c r="N25" s="51"/>
-      <c r="O25" s="51"/>
+      <c r="A25" s="28"/>
+      <c r="B25" s="28"/>
+      <c r="C25" s="28"/>
+      <c r="D25" s="28"/>
+      <c r="E25" s="28"/>
+      <c r="F25" s="28"/>
+      <c r="G25" s="28"/>
+      <c r="H25" s="28"/>
+      <c r="I25" s="28"/>
+      <c r="J25" s="28"/>
+      <c r="K25" s="28"/>
+      <c r="L25" s="28"/>
+      <c r="M25" s="28"/>
+      <c r="N25" s="28"/>
+      <c r="O25" s="28"/>
     </row>
     <row r="26" spans="1:15" s="4" customFormat="1" ht="18" customHeight="1">
-      <c r="A26" s="52" t="s">
+      <c r="A26" s="34" t="s">
         <v>55</v>
       </c>
-      <c r="B26" s="52"/>
-      <c r="C26" s="52"/>
-      <c r="D26" s="52"/>
-      <c r="E26" s="52"/>
-      <c r="F26" s="52"/>
-      <c r="G26" s="52"/>
-      <c r="H26" s="52"/>
-      <c r="I26" s="52"/>
-      <c r="J26" s="52"/>
-      <c r="K26" s="52"/>
-      <c r="L26" s="52"/>
-      <c r="M26" s="52"/>
-      <c r="N26" s="52"/>
-      <c r="O26" s="52"/>
+      <c r="B26" s="34"/>
+      <c r="C26" s="34"/>
+      <c r="D26" s="34"/>
+      <c r="E26" s="34"/>
+      <c r="F26" s="34"/>
+      <c r="G26" s="34"/>
+      <c r="H26" s="34"/>
+      <c r="I26" s="34"/>
+      <c r="J26" s="34"/>
+      <c r="K26" s="34"/>
+      <c r="L26" s="34"/>
+      <c r="M26" s="34"/>
+      <c r="N26" s="34"/>
+      <c r="O26" s="34"/>
     </row>
     <row r="27" spans="1:15" s="4" customFormat="1" ht="18" customHeight="1">
-      <c r="A27" s="51"/>
-      <c r="B27" s="51"/>
-      <c r="C27" s="51"/>
-      <c r="D27" s="51"/>
-      <c r="E27" s="51"/>
-      <c r="F27" s="51"/>
-      <c r="G27" s="51"/>
-      <c r="H27" s="51"/>
-      <c r="I27" s="51"/>
-      <c r="J27" s="51"/>
-      <c r="K27" s="51"/>
-      <c r="L27" s="51"/>
-      <c r="M27" s="51"/>
-      <c r="N27" s="51"/>
-      <c r="O27" s="51"/>
+      <c r="A27" s="28"/>
+      <c r="B27" s="28"/>
+      <c r="C27" s="28"/>
+      <c r="D27" s="28"/>
+      <c r="E27" s="28"/>
+      <c r="F27" s="28"/>
+      <c r="G27" s="28"/>
+      <c r="H27" s="28"/>
+      <c r="I27" s="28"/>
+      <c r="J27" s="28"/>
+      <c r="K27" s="28"/>
+      <c r="L27" s="28"/>
+      <c r="M27" s="28"/>
+      <c r="N27" s="28"/>
+      <c r="O27" s="28"/>
     </row>
     <row r="28" spans="1:15" s="4" customFormat="1" ht="18" customHeight="1">
-      <c r="A28" s="48" t="s">
+      <c r="A28" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="B28" s="49"/>
-      <c r="C28" s="49"/>
-      <c r="D28" s="49"/>
-      <c r="E28" s="49"/>
-      <c r="F28" s="49"/>
-      <c r="G28" s="49"/>
-      <c r="H28" s="49"/>
-      <c r="I28" s="49"/>
-      <c r="J28" s="49"/>
-      <c r="K28" s="49"/>
-      <c r="L28" s="49"/>
-      <c r="M28" s="49"/>
-      <c r="N28" s="49"/>
-      <c r="O28" s="49"/>
+      <c r="B28" s="32"/>
+      <c r="C28" s="32"/>
+      <c r="D28" s="32"/>
+      <c r="E28" s="32"/>
+      <c r="F28" s="32"/>
+      <c r="G28" s="32"/>
+      <c r="H28" s="32"/>
+      <c r="I28" s="32"/>
+      <c r="J28" s="32"/>
+      <c r="K28" s="32"/>
+      <c r="L28" s="32"/>
+      <c r="M28" s="32"/>
+      <c r="N28" s="32"/>
+      <c r="O28" s="32"/>
     </row>
     <row r="29" spans="1:15" s="4" customFormat="1" ht="64.5" customHeight="1">
       <c r="A29" s="1"/>
@@ -3177,19 +3157,19 @@
       <c r="D29" s="1"/>
       <c r="E29" s="1"/>
       <c r="F29" s="1"/>
-      <c r="G29" s="50"/>
-      <c r="H29" s="50"/>
-      <c r="I29" s="51" t="s">
+      <c r="G29" s="30"/>
+      <c r="H29" s="30"/>
+      <c r="I29" s="28" t="s">
         <v>32</v>
       </c>
-      <c r="J29" s="51"/>
-      <c r="K29" s="51"/>
-      <c r="L29" s="51"/>
-      <c r="M29" s="54" t="s">
+      <c r="J29" s="28"/>
+      <c r="K29" s="28"/>
+      <c r="L29" s="28"/>
+      <c r="M29" s="29" t="s">
         <v>57</v>
       </c>
-      <c r="N29" s="54"/>
-      <c r="O29" s="54"/>
+      <c r="N29" s="29"/>
+      <c r="O29" s="29"/>
     </row>
     <row r="30" spans="1:15" s="4" customFormat="1" ht="64.5" customHeight="1">
       <c r="A30" s="1"/>
@@ -3198,19 +3178,19 @@
       <c r="D30" s="1"/>
       <c r="E30" s="1"/>
       <c r="F30" s="1"/>
-      <c r="G30" s="50"/>
-      <c r="H30" s="50"/>
-      <c r="I30" s="51" t="s">
+      <c r="G30" s="30"/>
+      <c r="H30" s="30"/>
+      <c r="I30" s="28" t="s">
         <v>56</v>
       </c>
-      <c r="J30" s="51"/>
-      <c r="K30" s="51"/>
-      <c r="L30" s="51"/>
-      <c r="M30" s="54" t="s">
+      <c r="J30" s="28"/>
+      <c r="K30" s="28"/>
+      <c r="L30" s="28"/>
+      <c r="M30" s="29" t="s">
         <v>58</v>
       </c>
-      <c r="N30" s="54"/>
-      <c r="O30" s="54"/>
+      <c r="N30" s="29"/>
+      <c r="O30" s="29"/>
     </row>
     <row r="31" spans="1:15" s="4" customFormat="1" ht="18" customHeight="1">
       <c r="A31" s="1"/>
@@ -3219,15 +3199,15 @@
       <c r="D31" s="1"/>
       <c r="E31" s="1"/>
       <c r="F31" s="1"/>
-      <c r="G31" s="50"/>
-      <c r="H31" s="50"/>
-      <c r="I31" s="51"/>
-      <c r="J31" s="51"/>
-      <c r="K31" s="51"/>
-      <c r="L31" s="51"/>
-      <c r="M31" s="51"/>
-      <c r="N31" s="51"/>
-      <c r="O31" s="51"/>
+      <c r="G31" s="30"/>
+      <c r="H31" s="30"/>
+      <c r="I31" s="28"/>
+      <c r="J31" s="28"/>
+      <c r="K31" s="28"/>
+      <c r="L31" s="28"/>
+      <c r="M31" s="28"/>
+      <c r="N31" s="28"/>
+      <c r="O31" s="28"/>
     </row>
     <row r="32" spans="1:15" s="4" customFormat="1" ht="18" customHeight="1">
       <c r="A32" s="1"/>
@@ -3247,108 +3227,67 @@
       <c r="O32" s="21"/>
     </row>
     <row r="33" spans="1:15" ht="22.5" customHeight="1">
-      <c r="A33" s="24"/>
-      <c r="B33" s="24"/>
-      <c r="C33" s="24"/>
-      <c r="D33" s="24"/>
-      <c r="E33" s="24"/>
-      <c r="F33" s="24"/>
-      <c r="G33" s="24"/>
-      <c r="H33" s="24"/>
-      <c r="I33" s="24"/>
-      <c r="J33" s="24"/>
-      <c r="K33" s="24"/>
-      <c r="L33" s="24"/>
-      <c r="M33" s="24"/>
-      <c r="N33" s="24"/>
-      <c r="O33" s="24"/>
+      <c r="A33" s="26"/>
+      <c r="B33" s="26"/>
+      <c r="C33" s="26"/>
+      <c r="D33" s="26"/>
+      <c r="E33" s="26"/>
+      <c r="F33" s="26"/>
+      <c r="G33" s="26"/>
+      <c r="H33" s="26"/>
+      <c r="I33" s="26"/>
+      <c r="J33" s="26"/>
+      <c r="K33" s="26"/>
+      <c r="L33" s="26"/>
+      <c r="M33" s="26"/>
+      <c r="N33" s="26"/>
+      <c r="O33" s="26"/>
     </row>
     <row r="34" spans="1:15" ht="20.100000000000001" customHeight="1">
-      <c r="A34" s="53" t="s">
+      <c r="A34" s="27" t="s">
         <v>33</v>
       </c>
-      <c r="B34" s="53"/>
-      <c r="C34" s="53"/>
-      <c r="D34" s="53"/>
-      <c r="E34" s="53"/>
-      <c r="F34" s="53"/>
-      <c r="G34" s="53"/>
-      <c r="H34" s="53"/>
-      <c r="I34" s="53"/>
-      <c r="J34" s="53"/>
-      <c r="K34" s="53"/>
-      <c r="L34" s="53"/>
-      <c r="M34" s="53"/>
-      <c r="N34" s="53"/>
-      <c r="O34" s="53"/>
+      <c r="B34" s="27"/>
+      <c r="C34" s="27"/>
+      <c r="D34" s="27"/>
+      <c r="E34" s="27"/>
+      <c r="F34" s="27"/>
+      <c r="G34" s="27"/>
+      <c r="H34" s="27"/>
+      <c r="I34" s="27"/>
+      <c r="J34" s="27"/>
+      <c r="K34" s="27"/>
+      <c r="L34" s="27"/>
+      <c r="M34" s="27"/>
+      <c r="N34" s="27"/>
+      <c r="O34" s="27"/>
     </row>
     <row r="35" spans="1:15" ht="20.100000000000001" customHeight="1">
-      <c r="A35" s="51"/>
-      <c r="B35" s="51"/>
-      <c r="C35" s="51"/>
-      <c r="D35" s="51"/>
-      <c r="E35" s="51"/>
-      <c r="F35" s="51"/>
-      <c r="G35" s="51"/>
-      <c r="H35" s="51"/>
-      <c r="I35" s="51"/>
-      <c r="J35" s="51"/>
-      <c r="K35" s="51"/>
-      <c r="L35" s="51"/>
-      <c r="M35" s="51"/>
-      <c r="N35" s="51"/>
-      <c r="O35" s="51"/>
+      <c r="A35" s="28"/>
+      <c r="B35" s="28"/>
+      <c r="C35" s="28"/>
+      <c r="D35" s="28"/>
+      <c r="E35" s="28"/>
+      <c r="F35" s="28"/>
+      <c r="G35" s="28"/>
+      <c r="H35" s="28"/>
+      <c r="I35" s="28"/>
+      <c r="J35" s="28"/>
+      <c r="K35" s="28"/>
+      <c r="L35" s="28"/>
+      <c r="M35" s="28"/>
+      <c r="N35" s="28"/>
+      <c r="O35" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="70">
-    <mergeCell ref="A33:O33"/>
-    <mergeCell ref="A34:O34"/>
-    <mergeCell ref="A35:O35"/>
-    <mergeCell ref="M29:O29"/>
-    <mergeCell ref="M30:O30"/>
-    <mergeCell ref="I30:L30"/>
-    <mergeCell ref="G31:H31"/>
-    <mergeCell ref="I31:O31"/>
-    <mergeCell ref="A28:O28"/>
-    <mergeCell ref="G29:H29"/>
-    <mergeCell ref="G30:H30"/>
-    <mergeCell ref="I29:L29"/>
-    <mergeCell ref="A22:O22"/>
-    <mergeCell ref="A23:O23"/>
-    <mergeCell ref="A24:O24"/>
-    <mergeCell ref="A25:O25"/>
-    <mergeCell ref="A26:O26"/>
-    <mergeCell ref="A27:O27"/>
-    <mergeCell ref="A21:O21"/>
-    <mergeCell ref="B16:E16"/>
-    <mergeCell ref="F16:G16"/>
-    <mergeCell ref="H16:K16"/>
-    <mergeCell ref="L16:M16"/>
-    <mergeCell ref="B18:E18"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="H18:K18"/>
-    <mergeCell ref="L18:M18"/>
-    <mergeCell ref="B19:E19"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="H19:K19"/>
-    <mergeCell ref="L19:M19"/>
-    <mergeCell ref="A20:O20"/>
-    <mergeCell ref="B14:E14"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="H14:K14"/>
-    <mergeCell ref="L14:M14"/>
-    <mergeCell ref="B15:E15"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="H15:K15"/>
-    <mergeCell ref="L15:M15"/>
-    <mergeCell ref="B12:E12"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="H12:K12"/>
-    <mergeCell ref="L12:M12"/>
-    <mergeCell ref="B13:E13"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="H13:K13"/>
-    <mergeCell ref="L13:M13"/>
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A2:O2"/>
+    <mergeCell ref="C3:O3"/>
+    <mergeCell ref="C4:O4"/>
+    <mergeCell ref="C5:H5"/>
+    <mergeCell ref="I5:K5"/>
+    <mergeCell ref="M5:O5"/>
     <mergeCell ref="B11:E11"/>
     <mergeCell ref="F11:G11"/>
     <mergeCell ref="H11:K11"/>
@@ -3364,17 +3303,58 @@
     <mergeCell ref="L8:N8"/>
     <mergeCell ref="C9:O9"/>
     <mergeCell ref="A10:O10"/>
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A2:O2"/>
-    <mergeCell ref="C3:O3"/>
-    <mergeCell ref="C4:O4"/>
-    <mergeCell ref="C5:H5"/>
-    <mergeCell ref="I5:K5"/>
-    <mergeCell ref="M5:O5"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="H12:K12"/>
+    <mergeCell ref="L12:M12"/>
+    <mergeCell ref="B13:E13"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="H13:K13"/>
+    <mergeCell ref="L13:M13"/>
+    <mergeCell ref="B14:E14"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="H14:K14"/>
+    <mergeCell ref="L14:M14"/>
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="H15:K15"/>
+    <mergeCell ref="L15:M15"/>
+    <mergeCell ref="A21:O21"/>
+    <mergeCell ref="B16:E16"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="H16:K16"/>
+    <mergeCell ref="L16:M16"/>
+    <mergeCell ref="B18:E18"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="H18:K18"/>
+    <mergeCell ref="L18:M18"/>
+    <mergeCell ref="B19:E19"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="H19:K19"/>
+    <mergeCell ref="L19:M19"/>
+    <mergeCell ref="A20:O20"/>
+    <mergeCell ref="A28:O28"/>
+    <mergeCell ref="G29:H29"/>
+    <mergeCell ref="G30:H30"/>
+    <mergeCell ref="I29:L29"/>
+    <mergeCell ref="A22:O22"/>
+    <mergeCell ref="A23:O23"/>
+    <mergeCell ref="A24:O24"/>
+    <mergeCell ref="A25:O25"/>
+    <mergeCell ref="A26:O26"/>
+    <mergeCell ref="A27:O27"/>
+    <mergeCell ref="A33:O33"/>
+    <mergeCell ref="A34:O34"/>
+    <mergeCell ref="A35:O35"/>
+    <mergeCell ref="M29:O29"/>
+    <mergeCell ref="M30:O30"/>
+    <mergeCell ref="I30:L30"/>
+    <mergeCell ref="G31:H31"/>
+    <mergeCell ref="I31:O31"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.63" bottom="0.39370078740157483" header="0.51181102362204722" footer="0.44"/>
-  <pageSetup paperSize="9" scale="77" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="81" orientation="portrait" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
   <drawing r:id="rId2"/>
   <legacyDrawing r:id="rId3"/>

</xml_diff>